<commit_message>
Update reconstruction plan: add home.jsx analysis
home.jsx is unrouted dead code — /home route serves Dashboard.jsx.
Added to Sheet 1 (delete) and Sheet 2/5 clarify the /home flow.
Total delete list now 38 items; rewrite list 16 items.

https://claude.ai/code/session_01N6SGgHa5HJ3wwTBV7BGrQo
</commit_message>
<xml_diff>
--- a/MIS_Reconstruction_Plan.xlsx
+++ b/MIS_Reconstruction_Plan.xlsx
@@ -547,13 +547,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
@@ -581,7 +581,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Approve ✓</t>
+          <t>Approve</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -603,17 +603,17 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Components/RightSidebar.jsx</t>
+          <t>Pages/home.jsx  *** UNROUTED — dead code ***</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Home/Landing</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Duplicates left nav; rail buttons confusing — replace with top-bar actions</t>
+          <t>/home route serves Dashboard.jsx — home.jsx is not connected to ANY route. 181 lines with 2-sec artificial setTimeout, mixes attendance+tasks+orders. DELETE; Dashboard.jsx becomes the single home screen.</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr"/>
@@ -629,17 +629,17 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/FlowBuilderPage.jsx</t>
+          <t>Components/RightSidebar.jsx</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Automation</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Visual flow builder too complex; team of 4 has no time to design automations</t>
+          <t>Duplicates left nav; confusing rail buttons — move 5 actions to top navbar instead.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
@@ -655,17 +655,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/BankReconciliation.jsx</t>
+          <t>Pages/FlowBuilderPage.jsx</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Accounts</t>
+          <t>Automation</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Enterprise feature; wrong scale for 10 orders/day</t>
+          <t>Visual flow builder too complex; team of 4 has no time to design automations.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/TrialBalance.jsx</t>
+          <t>Pages/BankReconciliation.jsx</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Accountant-level tool; not needed daily</t>
+          <t>Enterprise feature; wrong scale for 10 orders/day.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr"/>
@@ -707,7 +707,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/OpeningBalance.jsx</t>
+          <t>Pages/TrialBalance.jsx</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -717,13 +717,13 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>One-time setup page; not needed after initial entry</t>
+          <t>Accountant-level tool; not needed daily.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -733,23 +733,23 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/GmailAccounts.jsx</t>
+          <t>Pages/OpeningBalance.jsx</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Accounts</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>WhatsApp covers all customer communication; Gmail adds complexity</t>
+          <t>One-time setup page; not needed after initial entry.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/EmailCompose.jsx</t>
+          <t>Pages/GmailAccounts.jsx</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Same — consolidated into WhatsApp</t>
+          <t>WhatsApp covers all customer communication; Gmail adds complexity.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
@@ -785,7 +785,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/EmailHistory.jsx</t>
+          <t>Pages/EmailCompose.jsx</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Same — consolidated into WhatsApp</t>
+          <t>Same — consolidated into WhatsApp.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr"/>
@@ -811,23 +811,23 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/CallLogs.jsx</t>
+          <t>Pages/EmailHistory.jsx</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Not core to printing business ops; rarely used</t>
+          <t>Same — consolidated into WhatsApp.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr"/>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -837,17 +837,17 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/DiaryUpload.jsx</t>
+          <t>Pages/CallLogs.jsx</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Non-essential daily upload feature</t>
+          <t>Not core to printing business ops; rarely used.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr"/>
@@ -863,17 +863,17 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/SopPage.jsx</t>
+          <t>Pages/DiaryUpload.jsx</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Ops</t>
+          <t>Misc</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Replace with simple daily checklist embedded in dashboard</t>
+          <t>Non-essential daily upload feature.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr"/>
@@ -889,23 +889,23 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/WorkflowTemplates.jsx</t>
+          <t>Pages/SopPage.jsx</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Automation</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Replaced by fixed pipeline; team doesn't need custom workflow editing</t>
+          <t>Replace with simple daily checklist embedded in dashboard.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr"/>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -915,23 +915,23 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/UpiPayment.jsx  (standalone)</t>
+          <t>Pages/WorkflowTemplates.jsx</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Accounts</t>
+          <t>Automation</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Merge UPI collection into dashboard quick-action widget instead</t>
+          <t>Replaced by fixed pipeline; team doesn't need custom workflow editing.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr"/>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/addTransaction1.jsx</t>
+          <t>Pages/UpiPayment.jsx  (standalone)</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Replace with inline quick-add in simple accounts log</t>
+          <t>Merge UPI collection into dashboard quick-action widget instead.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
@@ -967,23 +967,23 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/AttendanceReport.jsx  (duplicate)</t>
+          <t>Pages/addTransaction1.jsx</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Accounts</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Keep AllAttandance.jsx; remove duplicate report</t>
+          <t>Replace with inline quick-add in simple accounts log.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr"/>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -993,56 +993,56 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Pages/purchaseOrder.jsx</t>
+          <t>Pages/AttendanceReport.jsx  (duplicate)</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Overkill at current scale; add note on vendor payment instead</t>
+          <t>Keep AllAttandance.jsx; remove duplicate report.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr"/>
       <c r="F18" s="7" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Pages/purchaseOrder.jsx</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Overkill at current scale; add note on vendor payment instead.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶  Legacy WhatsApp (Baileys)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>MISFrontend/src/Pages/WhatsApp*.jsx  (Baileys pages)</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>WhatsApp</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Unofficial QR-based; fragile; Cloud API replaces it</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>High</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>MISFrontend/src/Components/whatsapp/ (legacy folder)</t>
+          <t>Pages/WhatsApp*.jsx  (all Baileys pages)</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>All legacy WA components; superseded by whatsappCloud/ folder</t>
+          <t>Unofficial QR-based; fragile; Cloud API replaces all of these.</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr"/>
@@ -1072,36 +1072,36 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▶  Reports — consolidate 17 → 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="3" t="n">
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Reports/allTransaction.jsx</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Reports</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>5 transaction views → 1 smart Collections report</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr"/>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Components/whatsapp/ (legacy folder)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>All legacy WA components; superseded by whatsappCloud/ folder.</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  Reports — consolidate 17 into 3</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Reports/allTransaction4D.jsx</t>
+          <t>Reports/allTransaction.jsx</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>5 transaction views collapse into 1 smart Collections report.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
@@ -1137,7 +1137,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Reports/allBills.jsx  (current 879-line version)</t>
+          <t>Reports/allTransaction4D.jsx</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Rebuild as simplified Bills tab inside Collections report</t>
+          <t>Same — fold into Collections report.</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr"/>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Reports/agingReport.jsx</t>
+          <t>Reports/allBills.jsx  (879-line version)</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -1173,13 +1173,13 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Overkill; receivables aging not actionable daily for small team</t>
+          <t>Rebuild as simplified Bills tab inside Collections report.</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr"/>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Reports/priorityReport.jsx</t>
+          <t>Reports/agingReport.jsx</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1199,13 +1199,13 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Admin-level; low daily use</t>
+          <t>Overkill; receivables aging not actionable daily for small team.</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr"/>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Reports/taskReport.jsx</t>
+          <t>Reports/priorityReport.jsx</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Tasks visible on dashboard; separate report not needed</t>
+          <t>Admin-level; low daily use.</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Reports/userReport.jsx</t>
+          <t>Reports/taskReport.jsx</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Admin-level; low daily use</t>
+          <t>Tasks visible on dashboard; separate report not needed.</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr"/>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Reports/allDelivery.jsx</t>
+          <t>Reports/userReport.jsx</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -1277,13 +1277,13 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Fold delivery tracking into Orders report</t>
+          <t>Admin-level; low daily use.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr"/>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1293,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Reports/billUpdate.jsx</t>
+          <t>Reports/allDelivery.jsx</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Bill status updates happen from Kanban; standalone page redundant</t>
+          <t>Fold delivery tracking into Orders report.</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr"/>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Reports/paymentReport.jsx</t>
+          <t>Reports/billUpdate.jsx</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Merge into Collections report</t>
+          <t>Bill status updates happen from Kanban; standalone page redundant.</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr"/>
@@ -1339,36 +1339,36 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▶  Backend</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="3" t="n">
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>MISBackend/src/routes/Baileys.js</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Remove with Baileys frontend</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr"/>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Reports/paymentReport.jsx</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Merge into Collections report.</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  Backend routes + models to remove</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>MISBackend/src/services/baileysService.js</t>
+          <t>MISBackend/routes/Baileys.js</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Remove with Baileys frontend.</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr"/>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>MISBackend/src/repositories/baileysAuthState.js</t>
+          <t>MISBackend/services/baileysService.js</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Same.</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr"/>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>MISBackend/src/routes/Gmail.js</t>
+          <t>MISBackend/repositories/baileysAuthState.js</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Remove with Gmail frontend</t>
+          <t>Same.</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr"/>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>MISBackend/src/routes/BankStatement.js</t>
+          <t>MISBackend/routes/Gmail.js</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Remove with BankReconciliation frontend</t>
+          <t>Remove with Gmail frontend.</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr"/>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>MISBackend/src/routes/workflowTemplate.js</t>
+          <t>MISBackend/routes/BankStatement.js</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Remove with WorkflowTemplates frontend</t>
+          <t>Remove with BankReconciliation frontend.</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr"/>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>MISBackend/src/routes/PurchaseOrder.js</t>
+          <t>MISBackend/routes/workflowTemplate.js</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -1518,13 +1518,13 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Remove with purchaseOrder frontend</t>
+          <t>Remove with WorkflowTemplates frontend.</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr"/>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>MISBackend/src/repositories/flow.js + flowSession.js</t>
+          <t>MISBackend/routes/PurchaseOrder.js</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
@@ -1544,26 +1544,52 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Remove with FlowBuilder frontend</t>
+          <t>Remove with purchaseOrder frontend.</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr"/>
       <c r="F41" s="7" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>MISBackend/repositories/flow.js + flowSession.js</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Remove with FlowBuilder frontend.</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A20:F20"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A23:F23"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"✅ Yes,⏭ Skip,❓ Later"</formula1>
+    <dataValidation sqref="E2:E42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,Skip,Later"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1576,14 +1602,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1616,7 +1642,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Approve ✓</t>
+          <t>Approve</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -1628,7 +1654,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ▶  NAVIGATION</t>
+          <t xml:space="preserve">  ▶  HOME / LANDING PAGE</t>
         </is>
       </c>
     </row>
@@ -1638,22 +1664,22 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Sidebar.jsx</t>
+          <t>Pages/home.jsx  →  DELETE (see Sheet 1 row 1)</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>288</t>
+          <t>181</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>~80</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>6 items flat list (Dashboard/Orders/Customers/Accounts/Reports/Settings); remove sidebarMenu.jsx config file</t>
+          <t>home.jsx is NOT the /home route — Dashboard.jsx is. home.jsx is dead code. After cleanup, ROUTES.HOME ('/home') continues to serve the new simplified Dashboard.jsx. No separate 'home' page needed.</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr"/>
@@ -1663,72 +1689,72 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="6" t="n">
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  NAVIGATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>TopNavbar.jsx</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Components/Sidebar.jsx</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>288</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>~80</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>6 items flat list: Dashboard / Orders / Customers / Accounts / Reports / Settings (admin only). Remove all groups and collapsible sections. Delete sidebarMenu.jsx config file entirely.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Components/TopNavbar.jsx</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>100+</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>~80</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Add [+ New Order] primary button; move 5 right-sidebar actions here; remove right sidebar dependency</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Footer.jsx  (mobile bottom nav)</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>~40</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>4 tabs: Dashboard / Orders / + New Order / Accounts; remove Tasks &amp; Chat tabs</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▶  DASHBOARD</t>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Add [+ New Order] primary button. Move 5 right-sidebar quick actions here. Remove right sidebar dependency.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1738,66 +1764,66 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Dashboard.jsx</t>
+          <t>Components/Footer.jsx  (mobile bottom nav)</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>50</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>~200</t>
+          <t>~40</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>5 KPI tiles (Today Orders, Ready, Overdue, Collected, Pending); Needs Attention list (max 5 stuck orders); Stage pipeline counts; remove resizable panels, customization drawer, attendance section, user tasks section</t>
+          <t>4 tabs only: Dashboard / Orders / + New Order / Accounts. Remove Tasks and Chat tabs.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="3" t="n">
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  DASHBOARD  (= the /home route)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Components/dashboard/ (folder)</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>~300</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>~80</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Keep SummaryCard + QuickActions; delete CrmSidebarPanel, ActionList, RoleWidget, DesignFilesWidget; simplify UpiCollectionSection to inline widget</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▶  ORDER MANAGEMENT</t>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Pages/Dashboard.jsx  — serves ROUTES.HOME = '/home'</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>754</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>~200</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>This IS the home screen after login. New layout: 5 KPI tiles (Today Orders, Ready, Overdue, Collected ₹, Pending ₹) + 'Needs Attention' list (max 5 stuck/overdue orders with [Move] button) + Stage pipeline count bar. REMOVE: resizable panels, customization drawer, attendance section, user tasks section, design files widget.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1807,22 +1833,22 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>addOrder1.jsx</t>
+          <t>Components/dashboard/  (folder)</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>1726</t>
+          <t>~300</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>~180</t>
+          <t>~80</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>6 fields: Customer autocomplete, Items/Qty/Rate table (max 5 rows), Due Date, Priority, Advance Paid, 2 save buttons (Enquiry / Order); remove vendor section, task groups, Drive integration, date override, WA toggle (always auto-send)</t>
+          <t>Keep SummaryCard + QuickActions only. Delete: CrmSidebarPanel, ActionList, RoleWidget, DesignFilesWidget. Simplify UpiCollectionSection to a single inline button.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr"/>
@@ -1832,72 +1858,72 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="3" t="n">
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  ORDER MANAGEMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>OrderUpdate.jsx</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Pages/addOrder1.jsx</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>1726</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>~180</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>6 fields only: Customer (autocomplete), Items/Qty/Rate table (max 5 rows), Due Date (default +3 days), Priority (Low/Normal/Urgent chip), Advance Paid (yes/no + amount). 2 save buttons: [Save as Enquiry] and [Save as Order]. REMOVE: vendor section (auto-assign on backend), task groups, Google Drive, date override, WA toggle (always auto-send).</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Pages/OrderUpdate.jsx</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>710</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>~150</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Read-only order detail; editable: due date, priority, items qty/rate, add note; stage advance moved to Kanban</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr"/>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>OrderKanban.jsx + OrderCard.jsx</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>~300</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>~150</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Keep Kanban paradigm; simplify card: customer, item summary, due date, amount, [→ Next Stage] button; remove drag-drop complexity; 8 columns = full pipeline</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▶  ACCOUNTS (Simplify)</t>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Read-only order detail. Editable fields: due date, priority, items qty/rate, add note. Stage advance moves to Kanban board only.</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1907,22 +1933,22 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>DayBook.jsx</t>
+          <t>Pages/OrderKanban.jsx + Components/orders/OrderCard.jsx</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>1066</t>
+          <t>~300</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>~120</t>
+          <t>~150</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Replace double-entry complexity with simple Income/Expense log: date, type, amount, category, note, linked order; auto-create income entry when order marked paid</t>
+          <t>Keep Kanban paradigm. Simpler card: #order · Customer | Item summary | Due: X days | ₹ amount | [→ Next Stage] button. 8 columns = full pipeline. Remove drag-drop; use [→ Stage] button only.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr"/>
@@ -1935,7 +1961,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ▶  REPORTS (Rebuild 3)</t>
+          <t xml:space="preserve">  ▶  ACCOUNTS  (Simplify)</t>
         </is>
       </c>
     </row>
@@ -1945,22 +1971,22 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Reports/allOrder.jsx  → Orders Report</t>
+          <t>Pages/DayBook.jsx</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>712</t>
+          <t>1066</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>~200</t>
+          <t>~120</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Table + filters: date range, stage, customer; Export Excel; replaces allOrder, AllOrderTableView, allDelivery</t>
+          <t>Replace double-entry complexity with Income/Expense log. Two tabs: Income (auto-created when order paid) | Expenses (manual). Table: Date | Type | Amount | Category | Order# | Note. Totals at top: Income ₹X — Expenses ₹Y = Profit ₹Z.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr"/>
@@ -1970,72 +1996,72 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="3" t="n">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  REPORTS  (Rebuild 17 → 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Reports/Collections Report  (new)</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Reports/allOrder.jsx  →  New: Orders Report</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>~200</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Table + filters: date range, stage, customer. Columns: Order# | Customer | Items | Amount | Stage | Due Date | Assigned. Export Excel. Replaces: allOrder, AllOrderTableView, allDelivery.</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>New file: Reports/collectionsReport.jsx</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>~200</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Income + expenses by date range; replaces allBills, allTransaction*, paymentReport</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Reports/customerReport.jsx</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>303</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>~150</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>Minor cleanup: remove unused columns; keep search, filter by group, edit/delete</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr"/>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▶  BACKEND</t>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Income + expenses by date. Summary: Total In | Total Out | Net. Replaces: allBills, allTransaction*, paymentReport. Export Excel.</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2045,105 +2071,144 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>orderLifecycleController.js</t>
+          <t>Reports/customerReport.jsx</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>~200</t>
+          <t>303</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>~180</t>
+          <t>~150</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Add auto-WhatsApp send after each stage change using existing whatsappCloudService.sendTemplate()</t>
+          <t>Minor cleanup: remove unused columns. Keep search, group filter, edit/delete.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="6" t="n">
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▶  BACKEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>messageScheduler.js</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>controllers/orderLifecycleController.js</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>~200</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>~180</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Add auto-WhatsApp send after each stage change using existing whatsappCloudService.sendTemplate(). Reuse whatsappTemplates.js config.</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>services/messageScheduler.js</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>~150</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>~200</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Add: (a) daily 10am payment reminder for delivered-unpaid orders; (b) 7pm owner summary via WhatsApp</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr"/>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Add two cron jobs: (a) daily 10am payment reminder for delivered-unpaid orders; (b) 7pm owner summary WhatsApp with today's stats.</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>App.jsx  (router)</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>66 routes</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>~35 routes</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Remove routes for deleted pages; keep active 35</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr"/>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Remove routes for all deleted pages. Keep ~35 active routes.</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A6:G6"/>
+  <mergeCells count="7">
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A4:G4"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A11:G11"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"✅ Yes,⏭ Skip,❓ Later"</formula1>
+    <dataValidation sqref="F2:F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,Skip,Later"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2161,9 +2226,9 @@
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
@@ -2196,7 +2261,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Approve ✓</t>
+          <t>Approve</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -2208,7 +2273,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ▶  WHATSAPP AUTO-MESSAGES (Backend)</t>
+          <t xml:space="preserve">  ▶  WHATSAPP AUTO-MESSAGES  (Backend — zero human action)</t>
         </is>
       </c>
     </row>
@@ -2218,22 +2283,22 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Stage-change WA message</t>
+          <t>Order confirmation WA</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Auto-send WA to customer when order moves to approved / design / ready / delivered</t>
+          <t>On order creation: auto-send 'Order #N received, amount Rs.X, due date Y' to customer.</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>orderLifecycleController.js + whatsappTemplates.js</t>
+          <t>orderService.js (create hook)</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Order stage PATCH</t>
+          <t>Order created</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr"/>
@@ -2249,22 +2314,22 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Payment reminder WA</t>
+          <t>Stage-change WA message</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Daily 10am: find delivered-unpaid orders older than 2 days → send WA payment due</t>
+          <t>Auto-send WA to customer when order moves to: approved / design / ready / delivered. Messages defined in whatsappTemplates.js.</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>messageScheduler.js</t>
+          <t>orderLifecycleController.js + whatsappTemplates.js</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Cron 10:00</t>
+          <t>PATCH /stage</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr"/>
@@ -2280,22 +2345,22 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Order confirmation WA</t>
+          <t>Payment reminder WA</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>On order creation: send 'Order #{n} received, amount ₹X, due date Y'</t>
+          <t>Daily 10am: find all delivered-unpaid orders older than 2 days. Send WA: 'Your order #N of Rs.X is pending payment.'</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>orderService.js (create)</t>
+          <t>messageScheduler.js</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Order created</t>
+          <t>Cron 10:00</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr"/>
@@ -2316,7 +2381,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>7pm every day: New orders, collections, pending, overdue count → WA to owner number</t>
+          <t>7pm every day: aggregate today's stats (new orders, stage moves, collections, overdue count). Send WhatsApp summary to owner's number (configured in BusinessOps).</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -2347,7 +2412,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>If enquiry stuck in 'quoted' stage &gt; 24h, auto-send follow-up</t>
+          <t>If enquiry stays in 'quoted' stage &gt; 24h, auto-send follow-up message to customer.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2357,7 +2422,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Cron daily</t>
+          <t>Cron daily 11:00</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr"/>
@@ -2370,7 +2435,7 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ▶  ORDER AUTOMATION (Backend)</t>
+          <t xml:space="preserve">  ▶  ORDER AUTOMATION  (Backend)</t>
         </is>
       </c>
     </row>
@@ -2385,12 +2450,12 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>On order creation, auto-assign vendor to each production step based on preferred vendor in Item master</t>
+          <t>On order creation, auto-assign preferred vendor to each production step based on item type — no manual vendor selection needed.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>orderService.js + vendorService.js</t>
+          <t>orderService.js + vendorService.js  (already exists, just not wired)</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -2416,7 +2481,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Auto-create designer task when order reaches 'design' stage (already partly built — wire up fully)</t>
+          <t>Auto-create designer task when order moves to 'design' stage. (Already partly built in orderLifecycleController — complete the wiring.)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -2442,22 +2507,22 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>SLA alert</t>
+          <t>SLA / stuck-order alert</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Flag order in dashboard 'Needs Attention' if stuck in same stage &gt; 2 days</t>
+          <t>Flag order in dashboard 'Needs Attention' section if it stays in the same stage &gt; 2 days.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Dashboard API + dashboard controller</t>
+          <t>dashboardSummaryController.js + /api/dashboard/stuck-orders endpoint</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Real-time check</t>
+          <t>Dashboard load</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr"/>
@@ -2485,7 +2550,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>When order marked 'paid', auto-create income transaction (no manual journal)</t>
+          <t>When order is marked 'paid', auto-create income transaction. No manual journal entry needed.</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -2511,17 +2576,17 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Auto invoice generate</t>
+          <t>Auto PDF invoice on delivery</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>On delivery (stage = delivered), auto-generate PDF invoice and attach to order</t>
+          <t>When stage moves to 'delivered', auto-generate PDF invoice and attach to order record.</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>orderLifecycleController.js + InvoiceModal.jsx</t>
+          <t>orderLifecycleController.js + InvoiceModal.jsx (existing)</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -2544,7 +2609,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="F2:F14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"✅ Yes,⏭ Skip,❓ Later"</formula1>
+      <formula1>"Yes,Skip,Later"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2561,9 +2626,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
@@ -2591,7 +2656,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Approve ✓</t>
+          <t>Approve</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -2623,7 +2688,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>All enquiries now stored as Orders with stage=enquiry; Enquiry table is dead</t>
+          <t>All enquiries now stored as Orders with stage=enquiry. Enquiry table is dead code.</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr"/>
@@ -2649,7 +2714,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Removing flow builder frontend; these collections unused</t>
+          <t>Removing flow builder frontend; collections unused.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
@@ -2675,7 +2740,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Removing Baileys WhatsApp; collections unused</t>
+          <t>Removing Baileys WhatsApp; collections unused.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
@@ -2701,7 +2766,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Removing Gmail integration</t>
+          <t>Removing Gmail integration.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr"/>
@@ -2727,7 +2792,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Removing bank reconciliation</t>
+          <t>Removing bank reconciliation.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
@@ -2753,7 +2818,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Removing purchase order module</t>
+          <t>Removing purchase order module.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
@@ -2779,7 +2844,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Removing call logs page</t>
+          <t>Removing call logs page.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
@@ -2805,7 +2870,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Removing diary upload</t>
+          <t>Removing diary upload.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr"/>
@@ -2838,7 +2903,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Legacy; replaced by Order.stage (string); every query must account for both — confusing</t>
+          <t>Legacy field; replaced by Order.stage (string). Every query must handle both — confusing and error-prone.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr"/>
@@ -2864,7 +2929,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Old FK; standardise to vendorUuid everywhere</t>
+          <t>Old FK; standardise to vendorUuid everywhere.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr"/>
@@ -2880,7 +2945,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Order.workflowSteps[]  (if empty for most orders)</t>
+          <t>Order.workflowSteps[]</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -2890,7 +2955,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Check if actively used; if &lt;20% orders have data, remove</t>
+          <t>Check if actively used; if fewer than 20% of orders have data, remove entirely.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr"/>
@@ -2923,7 +2988,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>/get-order-list is inconsistent; rename to /orders, /delivered-orders</t>
+          <t>Inconsistent with REST conventions; rename to /orders, /delivered-orders.</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
@@ -2949,7 +3014,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Mix of {success,message} and {status,message}; pick one schema</t>
+          <t>Mix of {success,message} and {status,message}; pick one schema and apply everywhere.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr"/>
@@ -2975,7 +3040,7 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Replace with null or first available user</t>
+          <t>Replace with null or first available user; hardcoded names break on new installs.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr"/>
@@ -3001,7 +3066,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Missing pagination causes slow load on large datasets</t>
+          <t>Missing pagination causes slow load; will get worse as order count grows.</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr"/>
@@ -3019,7 +3084,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="E2:E19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"✅ Yes,⏭ Skip,❓ Later"</formula1>
+      <formula1>"Yes,Skip,Later"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3035,8 +3100,8 @@
   <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -3053,227 +3118,227 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Approve ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="50" customHeight="1">
+          <t>Approve</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="55" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
+          <t>/home route  (= Dashboard.jsx)</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>After login, user lands on Dashboard.jsx served at ROUTES.HOME = '/home'. home.jsx (the unused file) is deleted. One home screen, no confusion.</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3" ht="55" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Dashboard — KPI Row</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>5 tiles in one row: Today Orders (blue) | Ready to Deliver (green) | Overdue (red, alert if &gt;0) | Collected Today Rs. (green) | Pending Payment Rs. (orange). Tap any tile to filter.</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Dashboard — Needs Attention</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Max 5 items. Each shows: order# + customer + current stage + days stuck + [Move Stage] button. Red background if overdue. Yellow if 1-2 days late. Empty state message: All on track!</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Dashboard — Stage Pipeline Bar</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Horizontal row: Enquiry(n) &gt; Quoted(n) &gt; Approved(n) &gt; Design(n) &gt; Printing(n) &gt; Post-Print(n) &gt; Ready(n) &gt; Delivered(n). Tap stage to filter Kanban.</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
           <t>Left Sidebar</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>6 items ONLY: Dashboard | Orders | Customers | Accounts | Reports | Settings (admin). Flat list, icon + label. No groups, no collapsible sections. Width 200px collapsed, 240px expanded.</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr"/>
-    </row>
-    <row r="3" ht="50" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>6 items ONLY: Dashboard | Orders | Customers | Accounts | Reports | Settings (admin). Flat list, icon + label. No groups, no collapsible sections. Width 200px.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Top Navbar</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Left: hamburger + logo. Center: page title. Right: [+ New Order] primary button + bell icon + user avatar.</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr"/>
-    </row>
-    <row r="4" ht="50" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Left: hamburger + logo. Center: page title. Right: [+ New Order] orange primary button + bell notification icon + user avatar.</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Right Sidebar</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>DELETE — replaced by top navbar actions</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr"/>
-    </row>
-    <row r="5" ht="50" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>DELETED — its 5 quick actions move to top navbar.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="55" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Mobile Bottom Nav</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>4 tabs: Dashboard | Orders | ➕ (add order) | Accounts. Sticky bottom. Remove Tasks &amp; Chat.</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6" ht="50" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>Dashboard — KPI Row</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>5 tiles in one row: Today Orders (blue) | Ready (green) | Overdue (red, alert) | Collected ₹ (green) | Pending ₹ (orange). Tap any tile → filter orders.</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
-    </row>
-    <row r="7" ht="50" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Dashboard — Needs Attention</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Max 5 items. Show: order# + customer + stage + days stuck + [→ Move] button. Red if overdue, yellow if 1-2 days. Empty state: ✅ All on track!</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8" ht="50" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Dashboard — Pipeline</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Horizontal stage count bar: Enquiry(n) → Quoted(n) → Approved(n) → Design(n) → Printing(n) → Post-Print(n) → Ready(n) → Delivered(n). Tap to filter kanban.</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9" ht="50" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>4 tabs: Dashboard | Orders | + (add order, prominent) | Accounts. Sticky bottom. Remove Tasks and Chat tabs.</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10" ht="55" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Add Order Form</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>6 fields: Customer (autocomplete), Item+Qty+Rate table (max 5 rows inline), Due Date (default +3 days), Priority (Low/Normal/Urgent chip), Advance Paid (yes/no + amount). Bottom: [Save as Enquiry] grey | [Save as Order] primary. No vendor section. No task groups.</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10" ht="50" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>6 fields: Customer (autocomplete search), Items+Qty+Rate inline table (max 5 rows), Due Date (datepicker, default today+3), Priority (Low/Normal/Urgent chip selector), Advance Paid (toggle yes/no + amount field). Bottom buttons: [Save as Enquiry] (grey outline) and [Save as Order] (primary orange).</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Kanban Board</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>8 columns matching all stages. Card: #number · Customer name | Item summary (1 line) | Due: X days | ₹ amount | [→ Stage] button. Click card = order detail modal. No drag-drop (buttons only for stage advance).</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11" ht="50" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>8 columns (all pipeline stages). Card shows: #N Customer | Item summary | Due: X days ago/from now | Rs. amount | [Next Stage] button. Tap card = order detail modal. No drag-drop — stage buttons only.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12" ht="55" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Order Detail Modal</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Read-only header (order#, customer, created date). Editable: due date, priority, note. Items table (edit qty/rate). Stage history timeline. [Mark Paid] button if delivered. [Print Invoice] button.</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12" ht="50" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Accounts / Income-Expense Log</t>
-        </is>
-      </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Two tabs: Income | Expenses. Simple table: Date | Category | Amount | Order# | Note. Top: totals — Income ₹X | Expenses ₹Y | Profit ₹Z. [+ Add Expense] button. Income auto-created from paid orders.</t>
+          <t>Header: order#, customer, created date (read-only). Editable: due date, priority, add note, items qty/rate. Bottom: stage history timeline. [Mark Paid] button (if stage=delivered). [Print Invoice] button.</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr"/>
     </row>
-    <row r="13" ht="50" customHeight="1">
+    <row r="13" ht="55" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
+          <t>Accounts Page</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Two tabs: Income | Expenses. Table: Date | Category | Amount | Order# | Note. Top summary bar: Income Rs.X — Expenses Rs.Y = Profit Rs.Z. [+ Add Expense] button. Income entries created automatically when order is paid.</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14" ht="55" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
           <t>Reports — Orders</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Filters: Date Range | Stage | Customer. Table columns: Order# | Customer | Items | Amount | Stage | Due Date | Assigned. Export Excel button.</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14" ht="50" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Filters: Date Range + Stage dropdown + Customer search. Table: Order# | Customer | Items | Amount | Stage | Due Date | Assigned To. Export Excel button top-right.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15" ht="55" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Reports — Collections</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Filters: Date Range | Type (Income/Expense). Summary: Total In | Total Out | Net. Table: Date | Type | Category | Amount | Order# | Note. Export Excel.</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr"/>
-    </row>
-    <row r="15" ht="50" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Notifications</t>
-        </is>
-      </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Bell icon in top navbar. Dropdown list: overdue orders, payment reminders, stage changes. Badge count. Mark all read.</t>
+          <t>Filters: Date Range + Type (Income/Expense). Summary row: Total In | Total Out | Net. Table: Date | Type | Category | Amount | Order# | Note. Export Excel.</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr"/>
     </row>
-    <row r="16" ht="50" customHeight="1">
+    <row r="16" ht="55" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
+          <t>Notifications Bell</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Dropdown list in top navbar: overdue orders, payment reminders, stage changes. Badge count. [Mark all read] button.</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
           <t>Colour Theme</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Primary: Deep blue #2C3E50. Accent: Orange #E67E22. Success: Green #27AE60. Danger: Red #C0392B. Background: #F8F9FA. Cards: White with subtle shadow.</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr"/>
-    </row>
-    <row r="17" ht="50" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Typography</t>
-        </is>
-      </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Headings: 600 weight, 16-20px. Body: 400 weight, 14px. Captions: 12px grey. Font: Inter or system-ui.</t>
+          <t>Primary: #2C3E50 (dark navy). Accent/CTA: #E67E22 (orange). Success: #27AE60. Danger: #C0392B. Background: #F8F9FA. Cards: white + subtle shadow.</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr"/>
     </row>
-    <row r="18" ht="50" customHeight="1">
+    <row r="18" ht="55" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Spacing / Density</t>
+          <t>Typography &amp; Spacing</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Comfortable density (not compact). Card padding 16px. Table row height 44px. Mobile tap targets min 44px.</t>
+          <t>Font: Inter or system-ui. Headings: 600 weight 16-20px. Body: 400 weight 14px. Captions: 12px grey. Card padding 16px. Table row height 44px. Mobile tap targets min 44px.</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr"/>
@@ -3281,7 +3346,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="C2:C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"✅ Yes,⏭ Skip,❓ Later"</formula1>
+      <formula1>"Yes,Skip,Later"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3298,12 +3363,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3334,7 +3399,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Approve ✓</t>
+          <t>Approve</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -3350,7 +3415,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="50" customHeight="1">
+    <row r="3" ht="55" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>1</t>
@@ -3363,12 +3428,12 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>~25 frontend pages, ~12 backend routes, ~8 DB models</t>
+          <t>~26 FE pages, ~12 BE routes, ~8 DB models</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Remove Baileys, Gmail, FlowBuilder, BankReconciliation, TrialBalance, CallLogs, DiaryUpload, legacy WA, 14 reports, SopPage, WorkflowTemplates, PurchaseOrder. Update App.jsx routes.</t>
+          <t>Delete home.jsx (unrouted). Remove Baileys, Gmail, FlowBuilder, BankReconciliation, TrialBalance, CallLogs, DiaryUpload, legacy WA pages/components, 14 reports, SopPage, WorkflowTemplates, PurchaseOrder. Update App.jsx routes.</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -3379,7 +3444,7 @@
       <c r="F3" s="5" t="inlineStr"/>
       <c r="G3" s="14" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -3390,7 +3455,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="50" customHeight="1">
+    <row r="5" ht="55" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>2</t>
@@ -3403,12 +3468,12 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Sidebar.jsx, TopNavbar.jsx, Footer.jsx, sidebarMenu.jsx (delete)</t>
+          <t>Sidebar.jsx, TopNavbar.jsx, Footer.jsx, delete sidebarMenu.jsx</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Flat 6-item sidebar, top quick-action bar, 4-tab mobile footer</t>
+          <t>Flat 6-item sidebar, top quick-action bar with [+ New Order], 4-tab mobile footer.</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -3419,18 +3484,18 @@
       <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="14" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ▶  Phase 3 — Dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="50" customHeight="1">
+          <t xml:space="preserve">  ▶  Phase 3 — Dashboard  (= /home)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>3</t>
@@ -3438,17 +3503,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Rebuild Dashboard</t>
+          <t>Rebuild Dashboard.jsx  (the /home route)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Dashboard.jsx, dashboard/ components folder</t>
+          <t>Dashboard.jsx, Components/dashboard/ folder</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>5 KPI tiles, Needs Attention section, Pipeline bar. Remove all panels/customization.</t>
+          <t>5 KPI tiles + Needs Attention list + Stage pipeline bar. Remove resizable panels, customization drawer, attendance section, user tasks section.</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -3459,7 +3524,7 @@
       <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3535,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="50" customHeight="1">
+    <row r="9" ht="55" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>4</t>
@@ -3488,7 +3553,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>6-field add order form, simplified edit form</t>
+          <t>6-field add order form. Simplified edit form (read-only + editable fields only).</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -3499,7 +3564,7 @@
       <c r="F9" s="5" t="inlineStr"/>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -3510,7 +3575,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="50" customHeight="1">
+    <row r="11" ht="55" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>5</t>
@@ -3528,7 +3593,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Simpler cards, [→ Stage] button, 8 columns, remove drag-drop</t>
+          <t>Simpler cards, [Next Stage] button, 8 columns, remove drag-drop.</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -3539,7 +3604,7 @@
       <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -3550,7 +3615,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="50" customHeight="1">
+    <row r="13" ht="55" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>6</t>
@@ -3558,7 +3623,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Rebuild Reports (17 → 3)</t>
+          <t>Rebuild Reports  (17 -&gt; 3)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -3568,7 +3633,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Orders Report, Collections Report, Customer Report</t>
+          <t>Orders Report, Collections Report (new file), Customer Report (minor cleanup).</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -3579,7 +3644,7 @@
       <c r="F13" s="5" t="inlineStr"/>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3655,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="50" customHeight="1">
+    <row r="15" ht="55" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>7</t>
@@ -3603,12 +3668,12 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>DayBook.jsx, Accounts routes</t>
+          <t>Pages/DayBook.jsx, accounts backend routes</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Replace with simple Income/Expense log</t>
+          <t>Replace double-entry DayBook with simple Income/Expense log. Two tabs.</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -3619,18 +3684,18 @@
       <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ▶  Phase 8 — Automation</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="50" customHeight="1">
+          <t xml:space="preserve">  ▶  Phase 8 — Backend Automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="55" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
           <t>8</t>
@@ -3638,17 +3703,17 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Add backend automation</t>
+          <t>Add automation</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>orderLifecycleController.js, messageScheduler.js, whatsappTemplates.js</t>
+          <t>orderLifecycleController.js, messageScheduler.js, whatsappTemplates.js, orderService.js</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Auto WA on stage change, payment reminders, daily owner summary, auto income entry</t>
+          <t>Auto WA on order creation + stage changes. Payment reminders cron (10am). Daily owner summary cron (7pm). Auto income entry on payment.</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -3659,7 +3724,7 @@
       <c r="F17" s="5" t="inlineStr"/>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -3670,7 +3735,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="50" customHeight="1">
+    <row r="19" ht="55" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>9</t>
@@ -3683,12 +3748,12 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>repositories/ folder, migration script</t>
+          <t>repositories/ folder + migration script</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Remove unused collections, remove Status[] array from Order model, add pagination</t>
+          <t>Remove unused collections (Enquiry, Flow, Baileys, Gmail, BankStatement, PurchaseOrder, CallLogs, DiaryDraft). Remove Order.Status[] array. Add pagination to /api/orders/all-data.</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -3699,7 +3764,7 @@
       <c r="F19" s="5" t="inlineStr"/>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3775,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="50" customHeight="1">
+    <row r="21" ht="55" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>10</t>
@@ -3728,7 +3793,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Test golden path: Create order → advance stages → verify WA sent → mark paid → check reports. Time it: target &lt;2 min order creation.</t>
+          <t>Golden path: Create order (target &lt;2 min) &gt; advance stages &gt; verify WA sent &gt; mark paid &gt; check collections report. Test mobile layout. Check role-based access.</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -3739,7 +3804,7 @@
       <c r="F21" s="5" t="inlineStr"/>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>⬜ Pending</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -3758,10 +3823,10 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="F2:F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"✅ Yes,⏭ Skip,❓ Later"</formula1>
+      <formula1>"Yes,Skip,Later"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"⬜ Pending,🔄 In Progress,✅ Done,⏸ On Hold"</formula1>
+      <formula1>"Pending,In Progress,Done,On Hold"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>